<commit_message>
Cambio en README + 2006.csv
</commit_message>
<xml_diff>
--- a/salidas/empresas/ABBV.xlsx
+++ b/salidas/empresas/ABBV.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensual" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EPS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acciones" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mensual" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="EPS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Acciones" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Info" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,13 +23,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +43,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,12 +51,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,58 +447,58 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>precio_ajustado</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>precio_cierre</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>volumen</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>eps_ttm</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>pe</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>acciones_circulacion</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>market_cap</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>rotacion</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>41305</v>
       </c>
       <c r="B2" t="n">
-        <v>21.58233451843262</v>
+        <v>21.58232879638672</v>
       </c>
       <c r="C2" t="n">
         <v>36.68999862670898</v>
@@ -501,11 +513,11 @@
       <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>41333</v>
       </c>
       <c r="B3" t="n">
-        <v>21.71762084960938</v>
+        <v>21.71761703491211</v>
       </c>
       <c r="C3" t="n">
         <v>36.91999816894531</v>
@@ -520,11 +532,11 @@
       <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>41364</v>
       </c>
       <c r="B4" t="n">
-        <v>23.98820114135742</v>
+        <v>23.98819732666016</v>
       </c>
       <c r="C4" t="n">
         <v>40.77999877929688</v>
@@ -539,11 +551,11 @@
       <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>41394</v>
       </c>
       <c r="B5" t="n">
-        <v>27.33889961242676</v>
+        <v>27.33890533447266</v>
       </c>
       <c r="C5" t="n">
         <v>46.04999923706055</v>
@@ -558,11 +570,11 @@
       <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>41425</v>
       </c>
       <c r="B6" t="n">
-        <v>25.34414291381836</v>
+        <v>25.34414100646973</v>
       </c>
       <c r="C6" t="n">
         <v>42.68999862670898</v>
@@ -583,11 +595,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>41455</v>
       </c>
       <c r="B7" t="n">
-        <v>24.54266548156738</v>
+        <v>24.54267120361328</v>
       </c>
       <c r="C7" t="n">
         <v>41.34000015258789</v>
@@ -608,11 +620,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>41486</v>
       </c>
       <c r="B8" t="n">
-        <v>27.24872779846191</v>
+        <v>27.24872398376465</v>
       </c>
       <c r="C8" t="n">
         <v>45.47999954223633</v>
@@ -633,11 +645,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>41517</v>
       </c>
       <c r="B9" t="n">
-        <v>25.52921295166016</v>
+        <v>25.52920913696289</v>
       </c>
       <c r="C9" t="n">
         <v>42.61000061035156</v>
@@ -658,11 +670,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>41547</v>
       </c>
       <c r="B10" t="n">
-        <v>26.79936981201172</v>
+        <v>26.79937934875488</v>
       </c>
       <c r="C10" t="n">
         <v>44.72999954223633</v>
@@ -683,11 +695,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>41578</v>
       </c>
       <c r="B11" t="n">
-        <v>29.28961181640625</v>
+        <v>29.28962516784668</v>
       </c>
       <c r="C11" t="n">
         <v>48.45000076293945</v>
@@ -708,11 +720,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>41608</v>
       </c>
       <c r="B12" t="n">
-        <v>29.28961181640625</v>
+        <v>29.28962516784668</v>
       </c>
       <c r="C12" t="n">
         <v>48.45000076293945</v>
@@ -733,11 +745,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>41639</v>
       </c>
       <c r="B13" t="n">
-        <v>31.92538642883301</v>
+        <v>31.92539405822754</v>
       </c>
       <c r="C13" t="n">
         <v>52.81000137329102</v>
@@ -758,11 +770,11 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>41670</v>
       </c>
       <c r="B14" t="n">
-        <v>29.99689483642578</v>
+        <v>29.99688720703125</v>
       </c>
       <c r="C14" t="n">
         <v>49.22999954223633</v>
@@ -783,11 +795,11 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>41698</v>
       </c>
       <c r="B15" t="n">
-        <v>31.02055931091309</v>
+        <v>31.02054595947266</v>
       </c>
       <c r="C15" t="n">
         <v>50.90999984741211</v>
@@ -812,11 +824,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>41729</v>
       </c>
       <c r="B16" t="n">
-        <v>31.3191089630127</v>
+        <v>31.31911849975586</v>
       </c>
       <c r="C16" t="n">
         <v>51.40000152587891</v>
@@ -841,11 +853,11 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>41759</v>
       </c>
       <c r="B17" t="n">
-        <v>32.01746368408203</v>
+        <v>32.01744842529297</v>
       </c>
       <c r="C17" t="n">
         <v>52.08000183105469</v>
@@ -870,7 +882,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>41790</v>
       </c>
       <c r="B18" t="n">
@@ -899,7 +911,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>41820</v>
       </c>
       <c r="B19" t="n">
@@ -928,11 +940,11 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>41851</v>
       </c>
       <c r="B20" t="n">
-        <v>32.4213752746582</v>
+        <v>32.42137908935547</v>
       </c>
       <c r="C20" t="n">
         <v>52.34000015258789</v>
@@ -957,11 +969,11 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>41882</v>
       </c>
       <c r="B21" t="n">
-        <v>34.24251556396484</v>
+        <v>34.24252319335938</v>
       </c>
       <c r="C21" t="n">
         <v>55.27999877929688</v>
@@ -986,11 +998,11 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>41912</v>
       </c>
       <c r="B22" t="n">
-        <v>35.77871322631836</v>
+        <v>35.77872467041016</v>
       </c>
       <c r="C22" t="n">
         <v>57.7599983215332</v>
@@ -1015,11 +1027,11 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>41943</v>
       </c>
       <c r="B23" t="n">
-        <v>39.6027717590332</v>
+        <v>39.60276794433594</v>
       </c>
       <c r="C23" t="n">
         <v>63.45999908447266</v>
@@ -1044,11 +1056,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>41973</v>
       </c>
       <c r="B24" t="n">
-        <v>43.18486785888672</v>
+        <v>43.18485641479492</v>
       </c>
       <c r="C24" t="n">
         <v>69.19999694824219</v>
@@ -1073,11 +1085,11 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>42004</v>
       </c>
       <c r="B25" t="n">
-        <v>40.83840560913086</v>
+        <v>40.83840179443359</v>
       </c>
       <c r="C25" t="n">
         <v>65.44000244140625</v>
@@ -1102,11 +1114,11 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>42035</v>
       </c>
       <c r="B26" t="n">
-        <v>37.9446907043457</v>
+        <v>37.94468688964844</v>
       </c>
       <c r="C26" t="n">
         <v>60.34999847412109</v>
@@ -1131,11 +1143,11 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>42063</v>
       </c>
       <c r="B27" t="n">
-        <v>38.03900909423828</v>
+        <v>38.03899383544922</v>
       </c>
       <c r="C27" t="n">
         <v>60.5</v>
@@ -1160,11 +1172,11 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>42094</v>
       </c>
       <c r="B28" t="n">
-        <v>36.80666732788086</v>
+        <v>36.80664825439453</v>
       </c>
       <c r="C28" t="n">
         <v>58.54000091552734</v>
@@ -1189,11 +1201,11 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>42124</v>
       </c>
       <c r="B29" t="n">
-        <v>40.99176406860352</v>
+        <v>40.99176025390625</v>
       </c>
       <c r="C29" t="n">
         <v>64.66000366210938</v>
@@ -1218,11 +1230,11 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>42155</v>
       </c>
       <c r="B30" t="n">
-        <v>42.21529769897461</v>
+        <v>42.21530151367188</v>
       </c>
       <c r="C30" t="n">
         <v>66.58999633789062</v>
@@ -1247,11 +1259,11 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>42185</v>
       </c>
       <c r="B31" t="n">
-        <v>42.59567642211914</v>
+        <v>42.59568786621094</v>
       </c>
       <c r="C31" t="n">
         <v>67.19000244140625</v>
@@ -1276,11 +1288,11 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>42216</v>
       </c>
       <c r="B32" t="n">
-        <v>44.71283340454102</v>
+        <v>44.71282958984375</v>
       </c>
       <c r="C32" t="n">
         <v>70.01000213623047</v>
@@ -1305,11 +1317,11 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>42247</v>
       </c>
       <c r="B33" t="n">
-        <v>39.85898971557617</v>
+        <v>39.85898590087891</v>
       </c>
       <c r="C33" t="n">
         <v>62.40999984741211</v>
@@ -1334,11 +1346,11 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>42277</v>
       </c>
       <c r="B34" t="n">
-        <v>34.74967956542969</v>
+        <v>34.74967575073242</v>
       </c>
       <c r="C34" t="n">
         <v>54.40999984741211</v>
@@ -1363,11 +1375,11 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>42308</v>
       </c>
       <c r="B35" t="n">
-        <v>38.38340759277344</v>
+        <v>38.38341903686523</v>
       </c>
       <c r="C35" t="n">
         <v>59.54999923706055</v>
@@ -1392,11 +1404,11 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>42338</v>
       </c>
       <c r="B36" t="n">
-        <v>37.48104095458984</v>
+        <v>37.48104476928711</v>
       </c>
       <c r="C36" t="n">
         <v>58.15000152587891</v>
@@ -1421,7 +1433,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>42369</v>
       </c>
       <c r="B37" t="n">
@@ -1450,11 +1462,11 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>42400</v>
       </c>
       <c r="B38" t="n">
-        <v>35.75788497924805</v>
+        <v>35.75788116455078</v>
       </c>
       <c r="C38" t="n">
         <v>54.90000152587891</v>
@@ -1479,7 +1491,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>42429</v>
       </c>
       <c r="B39" t="n">
@@ -1508,11 +1520,11 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>42460</v>
       </c>
       <c r="B40" t="n">
-        <v>37.20383071899414</v>
+        <v>37.20383453369141</v>
       </c>
       <c r="C40" t="n">
         <v>57.11999893188477</v>
@@ -1537,11 +1549,11 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>42490</v>
       </c>
       <c r="B41" t="n">
-        <v>40.11275100708008</v>
+        <v>40.11275482177734</v>
       </c>
       <c r="C41" t="n">
         <v>61</v>
@@ -1566,11 +1578,11 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>42521</v>
       </c>
       <c r="B42" t="n">
-        <v>41.38188171386719</v>
+        <v>41.38188552856445</v>
       </c>
       <c r="C42" t="n">
         <v>62.93000030517578</v>
@@ -1595,11 +1607,11 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>42551</v>
       </c>
       <c r="B43" t="n">
-        <v>40.71114730834961</v>
+        <v>40.71115493774414</v>
       </c>
       <c r="C43" t="n">
         <v>61.90999984741211</v>
@@ -1624,11 +1636,11 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>42582</v>
       </c>
       <c r="B44" t="n">
-        <v>43.93425750732422</v>
+        <v>43.93426513671875</v>
       </c>
       <c r="C44" t="n">
         <v>66.23000335693359</v>
@@ -1653,11 +1665,11 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>42613</v>
       </c>
       <c r="B45" t="n">
-        <v>42.52130126953125</v>
+        <v>42.52128982543945</v>
       </c>
       <c r="C45" t="n">
         <v>64.09999847412109</v>
@@ -1682,11 +1694,11 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>42643</v>
       </c>
       <c r="B46" t="n">
-        <v>41.83803939819336</v>
+        <v>41.83804321289062</v>
       </c>
       <c r="C46" t="n">
         <v>63.06999969482422</v>
@@ -1711,11 +1723,11 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>42674</v>
       </c>
       <c r="B47" t="n">
-        <v>37.34331893920898</v>
+        <v>37.34333038330078</v>
       </c>
       <c r="C47" t="n">
         <v>55.77999877929688</v>
@@ -1740,11 +1752,11 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>42704</v>
       </c>
       <c r="B48" t="n">
-        <v>40.70408248901367</v>
+        <v>40.70408630371094</v>
       </c>
       <c r="C48" t="n">
         <v>60.79999923706055</v>
@@ -1769,11 +1781,11 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>42735</v>
       </c>
       <c r="B49" t="n">
-        <v>41.92253875732422</v>
+        <v>41.92254257202148</v>
       </c>
       <c r="C49" t="n">
         <v>62.61999893188477</v>
@@ -1798,7 +1810,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>42766</v>
       </c>
       <c r="B50" t="n">
@@ -1827,7 +1839,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>42794</v>
       </c>
       <c r="B51" t="n">
@@ -1856,11 +1868,11 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>42825</v>
       </c>
       <c r="B52" t="n">
-        <v>44.06315612792969</v>
+        <v>44.06315994262695</v>
       </c>
       <c r="C52" t="n">
         <v>65.16000366210938</v>
@@ -1885,11 +1897,11 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>42855</v>
       </c>
       <c r="B53" t="n">
-        <v>45.03423309326172</v>
+        <v>45.03423690795898</v>
       </c>
       <c r="C53" t="n">
         <v>65.94000244140625</v>
@@ -1914,11 +1926,11 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>42886</v>
       </c>
       <c r="B54" t="n">
-        <v>45.0888671875</v>
+        <v>45.08886337280273</v>
       </c>
       <c r="C54" t="n">
         <v>66.01999664306641</v>
@@ -1943,7 +1955,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>42916</v>
       </c>
       <c r="B55" t="n">
@@ -1972,11 +1984,11 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>42947</v>
       </c>
       <c r="B56" t="n">
-        <v>48.17474746704102</v>
+        <v>48.17475128173828</v>
       </c>
       <c r="C56" t="n">
         <v>69.91000366210938</v>
@@ -2001,11 +2013,11 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>42978</v>
       </c>
       <c r="B57" t="n">
-        <v>51.88898849487305</v>
+        <v>51.88898086547852</v>
       </c>
       <c r="C57" t="n">
         <v>75.30000305175781</v>
@@ -2030,7 +2042,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>43008</v>
       </c>
       <c r="B58" t="n">
@@ -2059,11 +2071,11 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>43039</v>
       </c>
       <c r="B59" t="n">
-        <v>62.62482833862305</v>
+        <v>62.62484741210938</v>
       </c>
       <c r="C59" t="n">
         <v>90.25</v>
@@ -2088,11 +2100,11 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>43069</v>
       </c>
       <c r="B60" t="n">
-        <v>67.25316619873047</v>
+        <v>67.25318145751953</v>
       </c>
       <c r="C60" t="n">
         <v>96.91999816894531</v>
@@ -2117,11 +2129,11 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>43100</v>
       </c>
       <c r="B61" t="n">
-        <v>67.10745239257812</v>
+        <v>67.10746002197266</v>
       </c>
       <c r="C61" t="n">
         <v>96.70999908447266</v>
@@ -2146,11 +2158,11 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>43131</v>
       </c>
       <c r="B62" t="n">
-        <v>78.42848968505859</v>
+        <v>78.42848205566406</v>
       </c>
       <c r="C62" t="n">
         <v>112.2200012207031</v>
@@ -2175,7 +2187,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>43159</v>
       </c>
       <c r="B63" t="n">
@@ -2204,11 +2216,11 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>43190</v>
       </c>
       <c r="B64" t="n">
-        <v>66.14913177490234</v>
+        <v>66.14912414550781</v>
       </c>
       <c r="C64" t="n">
         <v>94.65000152587891</v>
@@ -2233,11 +2245,11 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>43220</v>
       </c>
       <c r="B65" t="n">
-        <v>68.17594146728516</v>
+        <v>68.17594909667969</v>
       </c>
       <c r="C65" t="n">
         <v>96.55000305175781</v>
@@ -2262,11 +2274,11 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>43251</v>
       </c>
       <c r="B66" t="n">
-        <v>69.86359405517578</v>
+        <v>69.86357879638672</v>
       </c>
       <c r="C66" t="n">
         <v>98.94000244140625</v>
@@ -2291,7 +2303,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>43281</v>
       </c>
       <c r="B67" t="n">
@@ -2320,11 +2332,11 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>43312</v>
       </c>
       <c r="B68" t="n">
-        <v>65.79063415527344</v>
+        <v>65.79064178466797</v>
       </c>
       <c r="C68" t="n">
         <v>92.23000335693359</v>
@@ -2349,11 +2361,11 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>43343</v>
       </c>
       <c r="B69" t="n">
-        <v>68.46562194824219</v>
+        <v>68.46560668945312</v>
       </c>
       <c r="C69" t="n">
         <v>95.98000335693359</v>
@@ -2378,11 +2390,11 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>43373</v>
       </c>
       <c r="B70" t="n">
-        <v>67.46695709228516</v>
+        <v>67.46694946289062</v>
       </c>
       <c r="C70" t="n">
         <v>94.58000183105469</v>
@@ -2407,11 +2419,11 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>43404</v>
       </c>
       <c r="B71" t="n">
-        <v>56.126953125</v>
+        <v>56.1269645690918</v>
       </c>
       <c r="C71" t="n">
         <v>77.84999847412109</v>
@@ -2436,11 +2448,11 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>43434</v>
       </c>
       <c r="B72" t="n">
-        <v>67.96518707275391</v>
+        <v>67.96519470214844</v>
       </c>
       <c r="C72" t="n">
         <v>94.26999664306641</v>
@@ -2465,11 +2477,11 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>43465</v>
       </c>
       <c r="B73" t="n">
-        <v>66.46559143066406</v>
+        <v>66.46560668945312</v>
       </c>
       <c r="C73" t="n">
         <v>92.19000244140625</v>
@@ -2494,11 +2506,11 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>43496</v>
       </c>
       <c r="B74" t="n">
-        <v>58.59607315063477</v>
+        <v>58.59610366821289</v>
       </c>
       <c r="C74" t="n">
         <v>80.29000091552734</v>
@@ -2523,11 +2535,11 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>43524</v>
       </c>
       <c r="B75" t="n">
-        <v>57.82981109619141</v>
+        <v>57.82981491088867</v>
       </c>
       <c r="C75" t="n">
         <v>79.23999786376953</v>
@@ -2552,11 +2564,11 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>43555</v>
       </c>
       <c r="B76" t="n">
-        <v>58.81502914428711</v>
+        <v>58.8150520324707</v>
       </c>
       <c r="C76" t="n">
         <v>80.58999633789062</v>
@@ -2581,11 +2593,11 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>43585</v>
       </c>
       <c r="B77" t="n">
-        <v>58.70748519897461</v>
+        <v>58.70749282836914</v>
       </c>
       <c r="C77" t="n">
         <v>79.38999938964844</v>
@@ -2610,11 +2622,11 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>43616</v>
       </c>
       <c r="B78" t="n">
-        <v>56.72568511962891</v>
+        <v>56.72566986083984</v>
       </c>
       <c r="C78" t="n">
         <v>76.70999908447266</v>
@@ -2639,11 +2651,11 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>43646</v>
       </c>
       <c r="B79" t="n">
-        <v>53.77513122558594</v>
+        <v>53.77513885498047</v>
       </c>
       <c r="C79" t="n">
         <v>72.72000122070312</v>
@@ -2668,11 +2680,11 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>43677</v>
       </c>
       <c r="B80" t="n">
-        <v>50.0155143737793</v>
+        <v>50.01550674438477</v>
       </c>
       <c r="C80" t="n">
         <v>66.62000274658203</v>
@@ -2697,11 +2709,11 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>43708</v>
       </c>
       <c r="B81" t="n">
-        <v>49.3548469543457</v>
+        <v>49.35485458374023</v>
       </c>
       <c r="C81" t="n">
         <v>65.73999786376953</v>
@@ -2726,11 +2738,11 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>43738</v>
       </c>
       <c r="B82" t="n">
-        <v>56.8474235534668</v>
+        <v>56.847412109375</v>
       </c>
       <c r="C82" t="n">
         <v>75.72000122070312</v>
@@ -2755,11 +2767,11 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>43769</v>
       </c>
       <c r="B83" t="n">
-        <v>60.59368515014648</v>
+        <v>60.59369659423828</v>
       </c>
       <c r="C83" t="n">
         <v>79.55000305175781</v>
@@ -2784,11 +2796,11 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>43799</v>
       </c>
       <c r="B84" t="n">
-        <v>66.82444000244141</v>
+        <v>66.82443237304688</v>
       </c>
       <c r="C84" t="n">
         <v>87.73000335693359</v>
@@ -2813,7 +2825,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>43830</v>
       </c>
       <c r="B85" t="n">
@@ -2842,11 +2854,11 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>43861</v>
       </c>
       <c r="B86" t="n">
-        <v>62.54715347290039</v>
+        <v>62.54716491699219</v>
       </c>
       <c r="C86" t="n">
         <v>81.01999664306641</v>
@@ -2871,11 +2883,11 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>43890</v>
       </c>
       <c r="B87" t="n">
-        <v>66.1678466796875</v>
+        <v>66.16783142089844</v>
       </c>
       <c r="C87" t="n">
         <v>85.70999908447266</v>
@@ -2900,11 +2912,11 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>43921</v>
       </c>
       <c r="B88" t="n">
-        <v>58.81841278076172</v>
+        <v>58.81842422485352</v>
       </c>
       <c r="C88" t="n">
         <v>76.19000244140625</v>
@@ -2929,11 +2941,11 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>43951</v>
       </c>
       <c r="B89" t="n">
-        <v>64.40451812744141</v>
+        <v>64.40453338623047</v>
       </c>
       <c r="C89" t="n">
         <v>82.19999694824219</v>
@@ -2958,11 +2970,11 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>43982</v>
       </c>
       <c r="B90" t="n">
-        <v>72.60789489746094</v>
+        <v>72.60788726806641</v>
       </c>
       <c r="C90" t="n">
         <v>92.66999816894531</v>
@@ -2987,7 +2999,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>44012</v>
       </c>
       <c r="B91" t="n">
@@ -3016,11 +3028,11 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>44043</v>
       </c>
       <c r="B92" t="n">
-        <v>75.27055358886719</v>
+        <v>75.27056884765625</v>
       </c>
       <c r="C92" t="n">
         <v>94.91000366210938</v>
@@ -3045,11 +3057,11 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" s="2" t="n">
         <v>44074</v>
       </c>
       <c r="B93" t="n">
-        <v>75.95259857177734</v>
+        <v>75.95258331298828</v>
       </c>
       <c r="C93" t="n">
         <v>95.76999664306641</v>
@@ -3074,11 +3086,11 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" s="2" t="n">
         <v>44104</v>
       </c>
       <c r="B94" t="n">
-        <v>69.46524810791016</v>
+        <v>69.46525573730469</v>
       </c>
       <c r="C94" t="n">
         <v>87.58999633789062</v>
@@ -3103,11 +3115,11 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" s="2" t="n">
         <v>44135</v>
       </c>
       <c r="B95" t="n">
-        <v>68.40959930419922</v>
+        <v>68.40959167480469</v>
       </c>
       <c r="C95" t="n">
         <v>85.09999847412109</v>
@@ -3132,11 +3144,11 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" s="2" t="n">
         <v>44165</v>
       </c>
       <c r="B96" t="n">
-        <v>84.06903839111328</v>
+        <v>84.06904602050781</v>
       </c>
       <c r="C96" t="n">
         <v>104.5800018310547</v>
@@ -3161,11 +3173,11 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" s="2" t="n">
         <v>44196</v>
       </c>
       <c r="B97" t="n">
-        <v>86.13500213623047</v>
+        <v>86.13499450683594</v>
       </c>
       <c r="C97" t="n">
         <v>107.1500015258789</v>
@@ -3190,11 +3202,11 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" s="2" t="n">
         <v>44227</v>
       </c>
       <c r="B98" t="n">
-        <v>83.34442901611328</v>
+        <v>83.34445190429688</v>
       </c>
       <c r="C98" t="n">
         <v>102.4800033569336</v>
@@ -3219,11 +3231,11 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" s="2" t="n">
         <v>44255</v>
       </c>
       <c r="B99" t="n">
-        <v>87.62226104736328</v>
+        <v>87.62226867675781</v>
       </c>
       <c r="C99" t="n">
         <v>107.7399978637695</v>
@@ -3248,11 +3260,11 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" s="2" t="n">
         <v>44286</v>
       </c>
       <c r="B100" t="n">
-        <v>88.01263427734375</v>
+        <v>88.01262664794922</v>
       </c>
       <c r="C100" t="n">
         <v>108.2200012207031</v>
@@ -3277,11 +3289,11 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" s="2" t="n">
         <v>44316</v>
       </c>
       <c r="B101" t="n">
-        <v>91.78272247314453</v>
+        <v>91.78271484375</v>
       </c>
       <c r="C101" t="n">
         <v>111.5</v>
@@ -3306,11 +3318,11 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" s="2" t="n">
         <v>44347</v>
       </c>
       <c r="B102" t="n">
-        <v>93.18207550048828</v>
+        <v>93.18208312988281</v>
       </c>
       <c r="C102" t="n">
         <v>113.1999969482422</v>
@@ -3335,11 +3347,11 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" s="2" t="n">
         <v>44377</v>
       </c>
       <c r="B103" t="n">
-        <v>92.72112274169922</v>
+        <v>92.72113037109375</v>
       </c>
       <c r="C103" t="n">
         <v>112.6399993896484</v>
@@ -3364,11 +3376,11 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" s="2" t="n">
         <v>44408</v>
       </c>
       <c r="B104" t="n">
-        <v>96.80117797851562</v>
+        <v>96.80115509033203</v>
       </c>
       <c r="C104" t="n">
         <v>116.3000030517578</v>
@@ -3393,11 +3405,11 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" s="2" t="n">
         <v>44439</v>
       </c>
       <c r="B105" t="n">
-        <v>100.5300674438477</v>
+        <v>100.5300598144531</v>
       </c>
       <c r="C105" t="n">
         <v>120.7799987792969</v>
@@ -3422,11 +3434,11 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" s="2" t="n">
         <v>44469</v>
       </c>
       <c r="B106" t="n">
-        <v>89.7845458984375</v>
+        <v>89.78455352783203</v>
       </c>
       <c r="C106" t="n">
         <v>107.870002746582</v>
@@ -3451,11 +3463,11 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" s="2" t="n">
         <v>44500</v>
       </c>
       <c r="B107" t="n">
-        <v>96.6015625</v>
+        <v>96.60157775878906</v>
       </c>
       <c r="C107" t="n">
         <v>114.6699981689453</v>
@@ -3480,7 +3492,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" s="2" t="n">
         <v>44530</v>
       </c>
       <c r="B108" t="n">
@@ -3509,11 +3521,11 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" s="2" t="n">
         <v>44561</v>
       </c>
       <c r="B109" t="n">
-        <v>114.0651550292969</v>
+        <v>114.0651702880859</v>
       </c>
       <c r="C109" t="n">
         <v>135.3999938964844</v>
@@ -3538,11 +3550,11 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" s="2" t="n">
         <v>44592</v>
       </c>
       <c r="B110" t="n">
-        <v>116.5170516967773</v>
+        <v>116.5170745849609</v>
       </c>
       <c r="C110" t="n">
         <v>136.8899993896484</v>
@@ -3567,11 +3579,11 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" s="2" t="n">
         <v>44620</v>
       </c>
       <c r="B111" t="n">
-        <v>125.7778549194336</v>
+        <v>125.7778701782227</v>
       </c>
       <c r="C111" t="n">
         <v>147.7700042724609</v>
@@ -3596,11 +3608,11 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" s="2" t="n">
         <v>44651</v>
       </c>
       <c r="B112" t="n">
-        <v>137.9836578369141</v>
+        <v>137.9836120605469</v>
       </c>
       <c r="C112" t="n">
         <v>162.1100006103516</v>
@@ -3625,11 +3637,11 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" s="2" t="n">
         <v>44681</v>
       </c>
       <c r="B113" t="n">
-        <v>126.0828170776367</v>
+        <v>126.0828552246094</v>
       </c>
       <c r="C113" t="n">
         <v>146.8800048828125</v>
@@ -3654,11 +3666,11 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" s="2" t="n">
         <v>44712</v>
       </c>
       <c r="B114" t="n">
-        <v>126.5034255981445</v>
+        <v>126.5034332275391</v>
       </c>
       <c r="C114" t="n">
         <v>147.3699951171875</v>
@@ -3683,11 +3695,11 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" s="2" t="n">
         <v>44742</v>
       </c>
       <c r="B115" t="n">
-        <v>131.4736328125</v>
+        <v>131.4736175537109</v>
       </c>
       <c r="C115" t="n">
         <v>153.1600036621094</v>
@@ -3712,11 +3724,11 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" s="2" t="n">
         <v>44773</v>
       </c>
       <c r="B116" t="n">
-        <v>124.34228515625</v>
+        <v>124.3422775268555</v>
       </c>
       <c r="C116" t="n">
         <v>143.5099945068359</v>
@@ -3741,11 +3753,11 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" s="2" t="n">
         <v>44804</v>
       </c>
       <c r="B117" t="n">
-        <v>116.5010299682617</v>
+        <v>116.5010375976562</v>
       </c>
       <c r="C117" t="n">
         <v>134.4600067138672</v>
@@ -3770,11 +3782,11 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" s="2" t="n">
         <v>44834</v>
       </c>
       <c r="B118" t="n">
-        <v>116.2844314575195</v>
+        <v>116.2844467163086</v>
       </c>
       <c r="C118" t="n">
         <v>134.2100067138672</v>
@@ -3799,11 +3811,11 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" s="2" t="n">
         <v>44865</v>
       </c>
       <c r="B119" t="n">
-        <v>128.1369934082031</v>
+        <v>128.1369781494141</v>
       </c>
       <c r="C119" t="n">
         <v>146.3999938964844</v>
@@ -3828,7 +3840,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" s="2" t="n">
         <v>44895</v>
       </c>
       <c r="B120" t="n">
@@ -3857,11 +3869,11 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" s="2" t="n">
         <v>44926</v>
       </c>
       <c r="B121" t="n">
-        <v>141.4495697021484</v>
+        <v>141.4496002197266</v>
       </c>
       <c r="C121" t="n">
         <v>161.6100006103516</v>
@@ -3886,11 +3898,11 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" s="2" t="n">
         <v>44957</v>
       </c>
       <c r="B122" t="n">
-        <v>130.5478973388672</v>
+        <v>130.5479278564453</v>
       </c>
       <c r="C122" t="n">
         <v>147.75</v>
@@ -3915,7 +3927,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" s="2" t="n">
         <v>44985</v>
       </c>
       <c r="B123" t="n">
@@ -3944,11 +3956,11 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" s="2" t="n">
         <v>45016</v>
       </c>
       <c r="B124" t="n">
-        <v>140.8150177001953</v>
+        <v>140.8150329589844</v>
       </c>
       <c r="C124" t="n">
         <v>159.3699951171875</v>
@@ -3973,7 +3985,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" s="2" t="n">
         <v>45046</v>
       </c>
       <c r="B125" t="n">
@@ -4002,11 +4014,11 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" s="2" t="n">
         <v>45077</v>
       </c>
       <c r="B126" t="n">
-        <v>123.0191192626953</v>
+        <v>123.0191345214844</v>
       </c>
       <c r="C126" t="n">
         <v>137.9600067138672</v>
@@ -4031,11 +4043,11 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" s="2" t="n">
         <v>45107</v>
       </c>
       <c r="B127" t="n">
-        <v>120.1389236450195</v>
+        <v>120.1389007568359</v>
       </c>
       <c r="C127" t="n">
         <v>134.7299957275391</v>
@@ -4060,11 +4072,11 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" s="2" t="n">
         <v>45138</v>
       </c>
       <c r="B128" t="n">
-        <v>134.8593597412109</v>
+        <v>134.8593444824219</v>
       </c>
       <c r="C128" t="n">
         <v>149.5800018310547</v>
@@ -4089,11 +4101,11 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" s="2" t="n">
         <v>45169</v>
       </c>
       <c r="B129" t="n">
-        <v>132.4972076416016</v>
+        <v>132.4971923828125</v>
       </c>
       <c r="C129" t="n">
         <v>146.9600067138672</v>
@@ -4118,7 +4130,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" s="2" t="n">
         <v>45199</v>
       </c>
       <c r="B130" t="n">
@@ -4147,11 +4159,11 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" s="2" t="n">
         <v>45230</v>
       </c>
       <c r="B131" t="n">
-        <v>128.56005859375</v>
+        <v>128.5600891113281</v>
       </c>
       <c r="C131" t="n">
         <v>141.1799926757812</v>
@@ -4176,11 +4188,11 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" s="2" t="n">
         <v>45260</v>
       </c>
       <c r="B132" t="n">
-        <v>129.6619567871094</v>
+        <v>129.6619415283203</v>
       </c>
       <c r="C132" t="n">
         <v>142.3899993896484</v>
@@ -4205,11 +4217,11 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" s="2" t="n">
         <v>45291</v>
       </c>
       <c r="B133" t="n">
-        <v>141.1174163818359</v>
+        <v>141.117431640625</v>
       </c>
       <c r="C133" t="n">
         <v>154.9700012207031</v>
@@ -4234,11 +4246,11 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" s="2" t="n">
         <v>45322</v>
       </c>
       <c r="B134" t="n">
-        <v>151.1348114013672</v>
+        <v>151.1347961425781</v>
       </c>
       <c r="C134" t="n">
         <v>164.3999938964844</v>
@@ -4263,11 +4275,11 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" s="2" t="n">
         <v>45351</v>
       </c>
       <c r="B135" t="n">
-        <v>161.8448181152344</v>
+        <v>161.8447875976562</v>
       </c>
       <c r="C135" t="n">
         <v>176.0500030517578</v>
@@ -4292,11 +4304,11 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" s="2" t="n">
         <v>45382</v>
       </c>
       <c r="B136" t="n">
-        <v>167.4066467285156</v>
+        <v>167.4066314697266</v>
       </c>
       <c r="C136" t="n">
         <v>182.1000061035156</v>
@@ -4321,7 +4333,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" s="2" t="n">
         <v>45412</v>
       </c>
       <c r="B137" t="n">
@@ -4350,11 +4362,11 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" s="2" t="n">
         <v>45443</v>
       </c>
       <c r="B138" t="n">
-        <v>149.6141052246094</v>
+        <v>149.6141204833984</v>
       </c>
       <c r="C138" t="n">
         <v>161.2400054931641</v>
@@ -4379,7 +4391,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" s="2" t="n">
         <v>45473</v>
       </c>
       <c r="B139" t="n">
@@ -4408,11 +4420,11 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" s="2" t="n">
         <v>45504</v>
       </c>
       <c r="B140" t="n">
-        <v>173.5375366210938</v>
+        <v>173.5375518798828</v>
       </c>
       <c r="C140" t="n">
         <v>185.3200073242188</v>
@@ -4437,7 +4449,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" s="2" t="n">
         <v>45535</v>
       </c>
       <c r="B141" t="n">
@@ -4466,7 +4478,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" s="2" t="n">
         <v>45565</v>
       </c>
       <c r="B142" t="n">
@@ -4495,11 +4507,11 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" s="2" t="n">
         <v>45596</v>
       </c>
       <c r="B143" t="n">
-        <v>192.4326171875</v>
+        <v>192.4326324462891</v>
       </c>
       <c r="C143" t="n">
         <v>203.8699951171875</v>
@@ -4524,11 +4536,11 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" s="2" t="n">
         <v>45626</v>
       </c>
       <c r="B144" t="n">
-        <v>172.6673889160156</v>
+        <v>172.6673736572266</v>
       </c>
       <c r="C144" t="n">
         <v>182.9299926757812</v>
@@ -4553,11 +4565,11 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" s="2" t="n">
         <v>45657</v>
       </c>
       <c r="B145" t="n">
-        <v>167.7308197021484</v>
+        <v>167.7308044433594</v>
       </c>
       <c r="C145" t="n">
         <v>177.6999969482422</v>
@@ -4582,11 +4594,11 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" s="2" t="n">
         <v>45688</v>
       </c>
       <c r="B146" t="n">
-        <v>175.2198791503906</v>
+        <v>175.2198944091797</v>
       </c>
       <c r="C146" t="n">
         <v>183.8999938964844</v>
@@ -4611,11 +4623,11 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" s="2" t="n">
         <v>45716</v>
       </c>
       <c r="B147" t="n">
-        <v>199.1637573242188</v>
+        <v>199.1637268066406</v>
       </c>
       <c r="C147" t="n">
         <v>209.0299987792969</v>
@@ -4640,7 +4652,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="B148" t="n">
@@ -4669,11 +4681,11 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" s="2" t="n">
         <v>45777</v>
       </c>
       <c r="B149" t="n">
-        <v>187.6091766357422</v>
+        <v>187.6091918945312</v>
       </c>
       <c r="C149" t="n">
         <v>195.1000061035156</v>
@@ -4698,7 +4710,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" s="2" t="n">
         <v>45808</v>
       </c>
       <c r="B150" t="n">
@@ -4727,11 +4739,11 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" s="2" t="n">
         <v>45838</v>
       </c>
       <c r="B151" t="n">
-        <v>178.4931335449219</v>
+        <v>178.4931640625</v>
       </c>
       <c r="C151" t="n">
         <v>185.6199951171875</v>
@@ -4756,7 +4768,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" s="2" t="n">
         <v>45869</v>
       </c>
       <c r="B152" t="n">
@@ -4785,11 +4797,11 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" s="2" t="n">
         <v>45900</v>
       </c>
       <c r="B153" t="n">
-        <v>204.0691833496094</v>
+        <v>204.0691986083984</v>
       </c>
       <c r="C153" t="n">
         <v>210.3999938964844</v>
@@ -4814,7 +4826,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="B154" t="n">
@@ -4843,7 +4855,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="B155" t="n">
@@ -4872,7 +4884,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" s="2" t="n">
         <v>45991</v>
       </c>
       <c r="B156" t="n">
@@ -4901,7 +4913,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" s="2" t="n">
         <v>46022</v>
       </c>
       <c r="B157" t="n">
@@ -4930,7 +4942,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" s="2" t="n">
         <v>46053</v>
       </c>
       <c r="B158" t="n">
@@ -4959,7 +4971,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" s="2" t="n">
         <v>46081</v>
       </c>
       <c r="B159" t="n">
@@ -4988,7 +5000,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="B160" t="n">
@@ -5017,7 +5029,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="B161" t="n">
@@ -5046,7 +5058,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" s="2" t="n">
         <v>46173</v>
       </c>
       <c r="B162" t="n">
@@ -5075,7 +5087,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="B163" t="n">
@@ -5104,7 +5116,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B164" t="n">
@@ -5133,7 +5145,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" s="2" t="n">
         <v>46265</v>
       </c>
       <c r="B165" t="n">
@@ -5162,32 +5174,32 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" s="2" t="n">
         <v>46295</v>
       </c>
       <c r="B166" t="n">
-        <v>265.0799865722656</v>
+        <v>265.1199951171875</v>
       </c>
       <c r="C166" t="n">
-        <v>265.0799865722656</v>
+        <v>265.1199951171875</v>
       </c>
       <c r="D166" t="n">
-        <v>67940600</v>
+        <v>71396600</v>
       </c>
       <c r="E166" t="n">
         <v>3.54</v>
       </c>
       <c r="F166" t="n">
-        <v>74.88135213905808</v>
+        <v>74.89265398790607</v>
       </c>
       <c r="G166" t="n">
         <v>1767117285</v>
       </c>
       <c r="H166" t="n">
-        <v>468427426179.4185</v>
+        <v>468498125970.6976</v>
       </c>
       <c r="I166" t="n">
-        <v>0.03844713680110939</v>
+        <v>0.04040286437467562</v>
       </c>
     </row>
   </sheetData>
@@ -5219,75 +5231,75 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>start</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>filed</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>form</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>fy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>fp</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>eps_trimestral</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>origen</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>eps_ttm</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>filed_ttm</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>factor</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>tag</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>40909</v>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>40999</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>41402</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -5323,13 +5335,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>41000</v>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>41090</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>41495</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -5365,13 +5377,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>41091</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>41182</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>41590</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -5407,13 +5419,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>41183</v>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>41274</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -5440,7 +5452,7 @@
       <c r="I5" t="n">
         <v>3.35</v>
       </c>
-      <c r="J5" s="1" t="n">
+      <c r="J5" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="K5" t="n">
@@ -5453,13 +5465,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>41275</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>41364</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>41402</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -5486,7 +5498,7 @@
       <c r="I6" t="n">
         <v>3.39</v>
       </c>
-      <c r="J6" s="1" t="n">
+      <c r="J6" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="K6" t="n">
@@ -5499,13 +5511,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>41365</v>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>41455</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>41495</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -5532,7 +5544,7 @@
       <c r="I7" t="n">
         <v>3.25</v>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J7" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="K7" t="n">
@@ -5545,13 +5557,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>41456</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>41547</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>41590</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -5578,7 +5590,7 @@
       <c r="I8" t="n">
         <v>2.84</v>
       </c>
-      <c r="J8" s="1" t="n">
+      <c r="J8" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="K8" t="n">
@@ -5591,13 +5603,13 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>41548</v>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>41639</v>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -5624,7 +5636,7 @@
       <c r="I9" t="n">
         <v>2.56</v>
       </c>
-      <c r="J9" s="1" t="n">
+      <c r="J9" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="K9" t="n">
@@ -5637,13 +5649,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>41640</v>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>41729</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>41768</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -5670,7 +5682,7 @@
       <c r="I10" t="n">
         <v>2.57</v>
       </c>
-      <c r="J10" s="1" t="n">
+      <c r="J10" s="2" t="n">
         <v>41768</v>
       </c>
       <c r="K10" t="n">
@@ -5683,13 +5695,13 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>41730</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>41820</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>41858</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -5716,7 +5728,7 @@
       <c r="I11" t="n">
         <v>2.59</v>
       </c>
-      <c r="J11" s="1" t="n">
+      <c r="J11" s="2" t="n">
         <v>41858</v>
       </c>
       <c r="K11" t="n">
@@ -5729,13 +5741,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>41821</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="n">
         <v>41912</v>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="2" t="n">
         <v>41950</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -5762,7 +5774,7 @@
       <c r="I12" t="n">
         <v>2.3</v>
       </c>
-      <c r="J12" s="1" t="n">
+      <c r="J12" s="2" t="n">
         <v>41950</v>
       </c>
       <c r="K12" t="n">
@@ -5775,13 +5787,13 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>41913</v>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B13" s="2" t="n">
         <v>42004</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="2" t="n">
         <v>42055</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -5808,7 +5820,7 @@
       <c r="I13" t="n">
         <v>1.09</v>
       </c>
-      <c r="J13" s="1" t="n">
+      <c r="J13" s="2" t="n">
         <v>42055</v>
       </c>
       <c r="K13" t="n">
@@ -5821,13 +5833,13 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>42005</v>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="2" t="n">
         <v>42094</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>42132</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -5854,7 +5866,7 @@
       <c r="I14" t="n">
         <v>1.11</v>
       </c>
-      <c r="J14" s="1" t="n">
+      <c r="J14" s="2" t="n">
         <v>42132</v>
       </c>
       <c r="K14" t="n">
@@ -5867,13 +5879,13 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>42095</v>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" s="2" t="n">
         <v>42185</v>
       </c>
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="2" t="n">
         <v>42223</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -5900,7 +5912,7 @@
       <c r="I15" t="n">
         <v>1.26</v>
       </c>
-      <c r="J15" s="1" t="n">
+      <c r="J15" s="2" t="n">
         <v>42223</v>
       </c>
       <c r="K15" t="n">
@@ -5913,13 +5925,13 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>42186</v>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="2" t="n">
         <v>42277</v>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>42314</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -5946,7 +5958,7 @@
       <c r="I16" t="n">
         <v>1.69</v>
       </c>
-      <c r="J16" s="1" t="n">
+      <c r="J16" s="2" t="n">
         <v>42314</v>
       </c>
       <c r="K16" t="n">
@@ -5959,13 +5971,13 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>42278</v>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" s="2" t="n">
         <v>42369</v>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>42419</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -5992,7 +6004,7 @@
       <c r="I17" t="n">
         <v>3.12</v>
       </c>
-      <c r="J17" s="1" t="n">
+      <c r="J17" s="2" t="n">
         <v>42419</v>
       </c>
       <c r="K17" t="n">
@@ -6005,13 +6017,13 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>42370</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="2" t="n">
         <v>42460</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="2" t="n">
         <v>42496</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -6038,7 +6050,7 @@
       <c r="I18" t="n">
         <v>3.32</v>
       </c>
-      <c r="J18" s="1" t="n">
+      <c r="J18" s="2" t="n">
         <v>42496</v>
       </c>
       <c r="K18" t="n">
@@ -6051,13 +6063,13 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>42461</v>
       </c>
-      <c r="B19" s="1" t="n">
+      <c r="B19" s="2" t="n">
         <v>42551</v>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C19" s="2" t="n">
         <v>42587</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -6084,7 +6096,7 @@
       <c r="I19" t="n">
         <v>3.47</v>
       </c>
-      <c r="J19" s="1" t="n">
+      <c r="J19" s="2" t="n">
         <v>42587</v>
       </c>
       <c r="K19" t="n">
@@ -6097,13 +6109,13 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>42552</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" s="2" t="n">
         <v>42643</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="2" t="n">
         <v>42681</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -6130,7 +6142,7 @@
       <c r="I20" t="n">
         <v>3.7</v>
       </c>
-      <c r="J20" s="1" t="n">
+      <c r="J20" s="2" t="n">
         <v>42681</v>
       </c>
       <c r="K20" t="n">
@@ -6143,13 +6155,13 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>42644</v>
       </c>
-      <c r="B21" s="1" t="n">
+      <c r="B21" s="2" t="n">
         <v>42735</v>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="2" t="n">
         <v>42783</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -6176,7 +6188,7 @@
       <c r="I21" t="n">
         <v>3.63</v>
       </c>
-      <c r="J21" s="1" t="n">
+      <c r="J21" s="2" t="n">
         <v>42783</v>
       </c>
       <c r="K21" t="n">
@@ -6189,13 +6201,13 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>42736</v>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" s="2" t="n">
         <v>42825</v>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="C22" s="2" t="n">
         <v>42860</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -6222,7 +6234,7 @@
       <c r="I22" t="n">
         <v>3.86</v>
       </c>
-      <c r="J22" s="1" t="n">
+      <c r="J22" s="2" t="n">
         <v>42860</v>
       </c>
       <c r="K22" t="n">
@@ -6235,13 +6247,13 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>42826</v>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" s="2" t="n">
         <v>42916</v>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="2" t="n">
         <v>42954</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -6268,7 +6280,7 @@
       <c r="I23" t="n">
         <v>4.07</v>
       </c>
-      <c r="J23" s="1" t="n">
+      <c r="J23" s="2" t="n">
         <v>42954</v>
       </c>
       <c r="K23" t="n">
@@ -6281,13 +6293,13 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>42917</v>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" s="2" t="n">
         <v>43008</v>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="2" t="n">
         <v>43046</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -6314,7 +6326,7 @@
       <c r="I24" t="n">
         <v>4.11</v>
       </c>
-      <c r="J24" s="1" t="n">
+      <c r="J24" s="2" t="n">
         <v>43046</v>
       </c>
       <c r="K24" t="n">
@@ -6327,13 +6339,13 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>43009</v>
       </c>
-      <c r="B25" s="1" t="n">
+      <c r="B25" s="2" t="n">
         <v>43100</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>43147</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -6360,7 +6372,7 @@
       <c r="I25" t="n">
         <v>3.29</v>
       </c>
-      <c r="J25" s="1" t="n">
+      <c r="J25" s="2" t="n">
         <v>43147</v>
       </c>
       <c r="K25" t="n">
@@ -6373,13 +6385,13 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>43101</v>
       </c>
-      <c r="B26" s="1" t="n">
+      <c r="B26" s="2" t="n">
         <v>43190</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>43224</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -6406,7 +6418,7 @@
       <c r="I26" t="n">
         <v>3.97</v>
       </c>
-      <c r="J26" s="1" t="n">
+      <c r="J26" s="2" t="n">
         <v>43224</v>
       </c>
       <c r="K26" t="n">
@@ -6419,13 +6431,13 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>43191</v>
       </c>
-      <c r="B27" s="1" t="n">
+      <c r="B27" s="2" t="n">
         <v>43281</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>43319</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -6452,7 +6464,7 @@
       <c r="I27" t="n">
         <v>4.04</v>
       </c>
-      <c r="J27" s="1" t="n">
+      <c r="J27" s="2" t="n">
         <v>43319</v>
       </c>
       <c r="K27" t="n">
@@ -6465,13 +6477,13 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>43282</v>
       </c>
-      <c r="B28" s="1" t="n">
+      <c r="B28" s="2" t="n">
         <v>43373</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>43411</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -6498,7 +6510,7 @@
       <c r="I28" t="n">
         <v>4.84</v>
       </c>
-      <c r="J28" s="1" t="n">
+      <c r="J28" s="2" t="n">
         <v>43411</v>
       </c>
       <c r="K28" t="n">
@@ -6511,13 +6523,13 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>43374</v>
       </c>
-      <c r="B29" s="1" t="n">
+      <c r="B29" s="2" t="n">
         <v>43465</v>
       </c>
-      <c r="C29" s="1" t="n">
+      <c r="C29" s="2" t="n">
         <v>43523</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -6544,7 +6556,7 @@
       <c r="I29" t="n">
         <v>3.58</v>
       </c>
-      <c r="J29" s="1" t="n">
+      <c r="J29" s="2" t="n">
         <v>43523</v>
       </c>
       <c r="K29" t="n">
@@ -6557,13 +6569,13 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>43466</v>
       </c>
-      <c r="B30" s="1" t="n">
+      <c r="B30" s="2" t="n">
         <v>43555</v>
       </c>
-      <c r="C30" s="1" t="n">
+      <c r="C30" s="2" t="n">
         <v>43588</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -6590,7 +6602,7 @@
       <c r="I30" t="n">
         <v>3.49</v>
       </c>
-      <c r="J30" s="1" t="n">
+      <c r="J30" s="2" t="n">
         <v>43588</v>
       </c>
       <c r="K30" t="n">
@@ -6603,13 +6615,13 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>43556</v>
       </c>
-      <c r="B31" s="1" t="n">
+      <c r="B31" s="2" t="n">
         <v>43646</v>
       </c>
-      <c r="C31" s="1" t="n">
+      <c r="C31" s="2" t="n">
         <v>43682</v>
       </c>
       <c r="D31" t="inlineStr">
@@ -6636,7 +6648,7 @@
       <c r="I31" t="n">
         <v>2.72</v>
       </c>
-      <c r="J31" s="1" t="n">
+      <c r="J31" s="2" t="n">
         <v>43682</v>
       </c>
       <c r="K31" t="n">
@@ -6649,13 +6661,13 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>43647</v>
       </c>
-      <c r="B32" s="1" t="n">
+      <c r="B32" s="2" t="n">
         <v>43738</v>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="C32" s="2" t="n">
         <v>43775</v>
       </c>
       <c r="D32" t="inlineStr">
@@ -6682,7 +6694,7 @@
       <c r="I32" t="n">
         <v>2.17</v>
       </c>
-      <c r="J32" s="1" t="n">
+      <c r="J32" s="2" t="n">
         <v>43775</v>
       </c>
       <c r="K32" t="n">
@@ -6695,13 +6707,13 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>43739</v>
       </c>
-      <c r="B33" s="1" t="n">
+      <c r="B33" s="2" t="n">
         <v>43830</v>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="2" t="n">
         <v>43882</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -6728,7 +6740,7 @@
       <c r="I33" t="n">
         <v>5.279999999999999</v>
       </c>
-      <c r="J33" s="1" t="n">
+      <c r="J33" s="2" t="n">
         <v>43882</v>
       </c>
       <c r="K33" t="n">
@@ -6741,13 +6753,13 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>43831</v>
       </c>
-      <c r="B34" s="1" t="n">
+      <c r="B34" s="2" t="n">
         <v>43921</v>
       </c>
-      <c r="C34" s="1" t="n">
+      <c r="C34" s="2" t="n">
         <v>43959</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -6774,7 +6786,7 @@
       <c r="I34" t="n">
         <v>5.65</v>
       </c>
-      <c r="J34" s="1" t="n">
+      <c r="J34" s="2" t="n">
         <v>43959</v>
       </c>
       <c r="K34" t="n">
@@ -6787,13 +6799,13 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>43922</v>
       </c>
-      <c r="B35" s="1" t="n">
+      <c r="B35" s="2" t="n">
         <v>44012</v>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="2" t="n">
         <v>44047</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -6820,7 +6832,7 @@
       <c r="I35" t="n">
         <v>4.699999999999999</v>
       </c>
-      <c r="J35" s="1" t="n">
+      <c r="J35" s="2" t="n">
         <v>44047</v>
       </c>
       <c r="K35" t="n">
@@ -6833,13 +6845,13 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>44013</v>
       </c>
-      <c r="B36" s="1" t="n">
+      <c r="B36" s="2" t="n">
         <v>44104</v>
       </c>
-      <c r="C36" s="1" t="n">
+      <c r="C36" s="2" t="n">
         <v>44139</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -6866,7 +6878,7 @@
       <c r="I36" t="n">
         <v>4.73</v>
       </c>
-      <c r="J36" s="1" t="n">
+      <c r="J36" s="2" t="n">
         <v>44139</v>
       </c>
       <c r="K36" t="n">
@@ -6879,13 +6891,13 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>44105</v>
       </c>
-      <c r="B37" s="1" t="n">
+      <c r="B37" s="2" t="n">
         <v>44196</v>
       </c>
-      <c r="C37" s="1" t="n">
+      <c r="C37" s="2" t="n">
         <v>44246</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -6912,7 +6924,7 @@
       <c r="I37" t="n">
         <v>2.86</v>
       </c>
-      <c r="J37" s="1" t="n">
+      <c r="J37" s="2" t="n">
         <v>44246</v>
       </c>
       <c r="K37" t="n">
@@ -6925,13 +6937,13 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>44197</v>
       </c>
-      <c r="B38" s="1" t="n">
+      <c r="B38" s="2" t="n">
         <v>44286</v>
       </c>
-      <c r="C38" s="1" t="n">
+      <c r="C38" s="2" t="n">
         <v>44323</v>
       </c>
       <c r="D38" t="inlineStr">
@@ -6958,7 +6970,7 @@
       <c r="I38" t="n">
         <v>2.83</v>
       </c>
-      <c r="J38" s="1" t="n">
+      <c r="J38" s="2" t="n">
         <v>44323</v>
       </c>
       <c r="K38" t="n">
@@ -6971,13 +6983,13 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>44287</v>
       </c>
-      <c r="B39" s="1" t="n">
+      <c r="B39" s="2" t="n">
         <v>44377</v>
       </c>
-      <c r="C39" s="1" t="n">
+      <c r="C39" s="2" t="n">
         <v>44410</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -7004,7 +7016,7 @@
       <c r="I39" t="n">
         <v>3.71</v>
       </c>
-      <c r="J39" s="1" t="n">
+      <c r="J39" s="2" t="n">
         <v>44410</v>
       </c>
       <c r="K39" t="n">
@@ -7017,13 +7029,13 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>44378</v>
       </c>
-      <c r="B40" s="1" t="n">
+      <c r="B40" s="2" t="n">
         <v>44469</v>
       </c>
-      <c r="C40" s="1" t="n">
+      <c r="C40" s="2" t="n">
         <v>44502</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -7050,7 +7062,7 @@
       <c r="I40" t="n">
         <v>4.2</v>
       </c>
-      <c r="J40" s="1" t="n">
+      <c r="J40" s="2" t="n">
         <v>44502</v>
       </c>
       <c r="K40" t="n">
@@ -7063,13 +7075,13 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>44470</v>
       </c>
-      <c r="B41" s="1" t="n">
+      <c r="B41" s="2" t="n">
         <v>44561</v>
       </c>
-      <c r="C41" s="1" t="n">
+      <c r="C41" s="2" t="n">
         <v>44610</v>
       </c>
       <c r="D41" t="inlineStr">
@@ -7096,7 +7108,7 @@
       <c r="I41" t="n">
         <v>6.45</v>
       </c>
-      <c r="J41" s="1" t="n">
+      <c r="J41" s="2" t="n">
         <v>44610</v>
       </c>
       <c r="K41" t="n">
@@ -7109,13 +7121,13 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>44562</v>
       </c>
-      <c r="B42" s="1" t="n">
+      <c r="B42" s="2" t="n">
         <v>44651</v>
       </c>
-      <c r="C42" s="1" t="n">
+      <c r="C42" s="2" t="n">
         <v>44687</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -7142,7 +7154,7 @@
       <c r="I42" t="n">
         <v>6.97</v>
       </c>
-      <c r="J42" s="1" t="n">
+      <c r="J42" s="2" t="n">
         <v>44687</v>
       </c>
       <c r="K42" t="n">
@@ -7155,13 +7167,13 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>44652</v>
       </c>
-      <c r="B43" s="1" t="n">
+      <c r="B43" s="2" t="n">
         <v>44742</v>
       </c>
-      <c r="C43" s="1" t="n">
+      <c r="C43" s="2" t="n">
         <v>44777</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -7188,7 +7200,7 @@
       <c r="I43" t="n">
         <v>7.06</v>
       </c>
-      <c r="J43" s="1" t="n">
+      <c r="J43" s="2" t="n">
         <v>44777</v>
       </c>
       <c r="K43" t="n">
@@ -7201,13 +7213,13 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>44743</v>
       </c>
-      <c r="B44" s="1" t="n">
+      <c r="B44" s="2" t="n">
         <v>44834</v>
       </c>
-      <c r="C44" s="1" t="n">
+      <c r="C44" s="2" t="n">
         <v>44869</v>
       </c>
       <c r="D44" t="inlineStr">
@@ -7234,7 +7246,7 @@
       <c r="I44" t="n">
         <v>7.489999999999999</v>
       </c>
-      <c r="J44" s="1" t="n">
+      <c r="J44" s="2" t="n">
         <v>44869</v>
       </c>
       <c r="K44" t="n">
@@ -7247,13 +7259,13 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>44835</v>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="B45" s="2" t="n">
         <v>44926</v>
       </c>
-      <c r="C45" s="1" t="n">
+      <c r="C45" s="2" t="n">
         <v>44974</v>
       </c>
       <c r="D45" t="inlineStr">
@@ -7280,7 +7292,7 @@
       <c r="I45" t="n">
         <v>6.609999999999999</v>
       </c>
-      <c r="J45" s="1" t="n">
+      <c r="J45" s="2" t="n">
         <v>44974</v>
       </c>
       <c r="K45" t="n">
@@ -7293,13 +7305,13 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>44927</v>
       </c>
-      <c r="B46" s="1" t="n">
+      <c r="B46" s="2" t="n">
         <v>45016</v>
       </c>
-      <c r="C46" s="1" t="n">
+      <c r="C46" s="2" t="n">
         <v>45051</v>
       </c>
       <c r="D46" t="inlineStr">
@@ -7326,7 +7338,7 @@
       <c r="I46" t="n">
         <v>4.23</v>
       </c>
-      <c r="J46" s="1" t="n">
+      <c r="J46" s="2" t="n">
         <v>45051</v>
       </c>
       <c r="K46" t="n">
@@ -7339,13 +7351,13 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>45017</v>
       </c>
-      <c r="B47" s="1" t="n">
+      <c r="B47" s="2" t="n">
         <v>45107</v>
       </c>
-      <c r="C47" s="1" t="n">
+      <c r="C47" s="2" t="n">
         <v>45145</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -7372,7 +7384,7 @@
       <c r="I47" t="n">
         <v>4.859999999999999</v>
       </c>
-      <c r="J47" s="1" t="n">
+      <c r="J47" s="2" t="n">
         <v>45145</v>
       </c>
       <c r="K47" t="n">
@@ -7385,13 +7397,13 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>45108</v>
       </c>
-      <c r="B48" s="1" t="n">
+      <c r="B48" s="2" t="n">
         <v>45199</v>
       </c>
-      <c r="C48" s="1" t="n">
+      <c r="C48" s="2" t="n">
         <v>45236</v>
       </c>
       <c r="D48" t="inlineStr">
@@ -7418,7 +7430,7 @@
       <c r="I48" t="n">
         <v>3.65</v>
       </c>
-      <c r="J48" s="1" t="n">
+      <c r="J48" s="2" t="n">
         <v>45236</v>
       </c>
       <c r="K48" t="n">
@@ -7431,13 +7443,13 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>45200</v>
       </c>
-      <c r="B49" s="1" t="n">
+      <c r="B49" s="2" t="n">
         <v>45291</v>
       </c>
-      <c r="C49" s="1" t="n">
+      <c r="C49" s="2" t="n">
         <v>45342</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -7464,7 +7476,7 @@
       <c r="I49" t="n">
         <v>2.73</v>
       </c>
-      <c r="J49" s="1" t="n">
+      <c r="J49" s="2" t="n">
         <v>45342</v>
       </c>
       <c r="K49" t="n">
@@ -7477,13 +7489,13 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>45292</v>
       </c>
-      <c r="B50" s="1" t="n">
+      <c r="B50" s="2" t="n">
         <v>45382</v>
       </c>
-      <c r="C50" s="1" t="n">
+      <c r="C50" s="2" t="n">
         <v>45415</v>
       </c>
       <c r="D50" t="inlineStr">
@@ -7510,7 +7522,7 @@
       <c r="I50" t="n">
         <v>3.37</v>
       </c>
-      <c r="J50" s="1" t="n">
+      <c r="J50" s="2" t="n">
         <v>45415</v>
       </c>
       <c r="K50" t="n">
@@ -7523,13 +7535,13 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="B51" s="1" t="n">
+      <c r="B51" s="2" t="n">
         <v>45473</v>
       </c>
-      <c r="C51" s="1" t="n">
+      <c r="C51" s="2" t="n">
         <v>45511</v>
       </c>
       <c r="D51" t="inlineStr">
@@ -7556,7 +7568,7 @@
       <c r="I51" t="n">
         <v>3</v>
       </c>
-      <c r="J51" s="1" t="n">
+      <c r="J51" s="2" t="n">
         <v>45511</v>
       </c>
       <c r="K51" t="n">
@@ -7569,13 +7581,13 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>45474</v>
       </c>
-      <c r="B52" s="1" t="n">
+      <c r="B52" s="2" t="n">
         <v>45565</v>
       </c>
-      <c r="C52" s="1" t="n">
+      <c r="C52" s="2" t="n">
         <v>45600</v>
       </c>
       <c r="D52" t="inlineStr">
@@ -7602,7 +7614,7 @@
       <c r="I52" t="n">
         <v>2.88</v>
       </c>
-      <c r="J52" s="1" t="n">
+      <c r="J52" s="2" t="n">
         <v>45600</v>
       </c>
       <c r="K52" t="n">
@@ -7615,13 +7627,13 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>45566</v>
       </c>
-      <c r="B53" s="1" t="n">
+      <c r="B53" s="2" t="n">
         <v>45657</v>
       </c>
-      <c r="C53" s="1" t="n">
+      <c r="C53" s="2" t="n">
         <v>45702</v>
       </c>
       <c r="D53" t="inlineStr">
@@ -7648,7 +7660,7 @@
       <c r="I53" t="n">
         <v>2.4</v>
       </c>
-      <c r="J53" s="1" t="n">
+      <c r="J53" s="2" t="n">
         <v>45702</v>
       </c>
       <c r="K53" t="n">
@@ -7661,13 +7673,13 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>45658</v>
       </c>
-      <c r="B54" s="1" t="n">
+      <c r="B54" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="C54" s="1" t="n">
+      <c r="C54" s="2" t="n">
         <v>45786</v>
       </c>
       <c r="D54" t="inlineStr">
@@ -7694,7 +7706,7 @@
       <c r="I54" t="n">
         <v>2.35</v>
       </c>
-      <c r="J54" s="1" t="n">
+      <c r="J54" s="2" t="n">
         <v>45786</v>
       </c>
       <c r="K54" t="n">
@@ -7707,13 +7719,13 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="B55" s="1" t="n">
+      <c r="B55" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="C55" s="1" t="n">
+      <c r="C55" s="2" t="n">
         <v>45873</v>
       </c>
       <c r="D55" t="inlineStr">
@@ -7740,7 +7752,7 @@
       <c r="I55" t="n">
         <v>2.1</v>
       </c>
-      <c r="J55" s="1" t="n">
+      <c r="J55" s="2" t="n">
         <v>45873</v>
       </c>
       <c r="K55" t="n">
@@ -7753,13 +7765,13 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="B56" s="1" t="n">
+      <c r="B56" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="C56" s="1" t="n">
+      <c r="C56" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="D56" t="inlineStr">
@@ -7786,7 +7798,7 @@
       <c r="I56" t="n">
         <v>1.32</v>
       </c>
-      <c r="J56" s="1" t="n">
+      <c r="J56" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="K56" t="n">
@@ -7799,13 +7811,13 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="B57" s="1" t="n">
+      <c r="B57" s="2" t="n">
         <v>46022</v>
       </c>
-      <c r="C57" s="1" t="n">
+      <c r="C57" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="D57" t="inlineStr">
@@ -7832,7 +7844,7 @@
       <c r="I57" t="n">
         <v>2.36</v>
       </c>
-      <c r="J57" s="1" t="n">
+      <c r="J57" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="K57" t="n">
@@ -7845,13 +7857,13 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>46023</v>
       </c>
-      <c r="B58" s="1" t="n">
+      <c r="B58" s="2" t="n">
         <v>46112</v>
       </c>
-      <c r="C58" s="1" t="n">
+      <c r="C58" s="2" t="n">
         <v>46150</v>
       </c>
       <c r="D58" t="inlineStr">
@@ -7878,7 +7890,7 @@
       <c r="I58" t="n">
         <v>2.03</v>
       </c>
-      <c r="J58" s="1" t="n">
+      <c r="J58" s="2" t="n">
         <v>46150</v>
       </c>
       <c r="K58" t="n">
@@ -7891,13 +7903,13 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>46113</v>
       </c>
-      <c r="B59" s="1" t="n">
+      <c r="B59" s="2" t="n">
         <v>46203</v>
       </c>
-      <c r="C59" s="1" t="n">
+      <c r="C59" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="D59" t="inlineStr">
@@ -7924,7 +7936,7 @@
       <c r="I59" t="n">
         <v>3.54</v>
       </c>
-      <c r="J59" s="1" t="n">
+      <c r="J59" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="K59" t="n">
@@ -7961,52 +7973,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>end</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>filed</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>acciones</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>form</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>fy</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>fp</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>tag</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>factor</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>41364</v>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
         <v>41402</v>
       </c>
       <c r="C2" t="n">
@@ -8035,10 +8047,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>41455</v>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
         <v>41495</v>
       </c>
       <c r="C3" t="n">
@@ -8067,10 +8079,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>41547</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
         <v>41590</v>
       </c>
       <c r="C4" t="n">
@@ -8099,10 +8111,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>41670</v>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
         <v>41691</v>
       </c>
       <c r="C5" t="n">
@@ -8131,10 +8143,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>41729</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>41768</v>
       </c>
       <c r="C6" t="n">
@@ -8163,10 +8175,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>41820</v>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
         <v>41858</v>
       </c>
       <c r="C7" t="n">
@@ -8195,10 +8207,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>41912</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
         <v>41950</v>
       </c>
       <c r="C8" t="n">
@@ -8227,10 +8239,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>42035</v>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
         <v>42055</v>
       </c>
       <c r="C9" t="n">
@@ -8259,10 +8271,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>42094</v>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
         <v>42132</v>
       </c>
       <c r="C10" t="n">
@@ -8291,10 +8303,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>42185</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>42223</v>
       </c>
       <c r="C11" t="n">
@@ -8323,10 +8335,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>42277</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="n">
         <v>42314</v>
       </c>
       <c r="C12" t="n">
@@ -8355,10 +8367,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>42400</v>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B13" s="2" t="n">
         <v>42419</v>
       </c>
       <c r="C13" t="n">
@@ -8387,10 +8399,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>42460</v>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="2" t="n">
         <v>42496</v>
       </c>
       <c r="C14" t="n">
@@ -8419,10 +8431,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>42551</v>
       </c>
-      <c r="B15" s="1" t="n">
+      <c r="B15" s="2" t="n">
         <v>42587</v>
       </c>
       <c r="C15" t="n">
@@ -8451,10 +8463,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>42667</v>
       </c>
-      <c r="B16" s="1" t="n">
+      <c r="B16" s="2" t="n">
         <v>42681</v>
       </c>
       <c r="C16" t="n">
@@ -8483,10 +8495,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>42766</v>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B17" s="2" t="n">
         <v>42783</v>
       </c>
       <c r="C17" t="n">
@@ -8515,10 +8527,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>42849</v>
       </c>
-      <c r="B18" s="1" t="n">
+      <c r="B18" s="2" t="n">
         <v>42860</v>
       </c>
       <c r="C18" t="n">
@@ -8547,10 +8559,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>42940</v>
       </c>
-      <c r="B19" s="1" t="n">
+      <c r="B19" s="2" t="n">
         <v>42954</v>
       </c>
       <c r="C19" t="n">
@@ -8579,10 +8591,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>43032</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B20" s="2" t="n">
         <v>43046</v>
       </c>
       <c r="C20" t="n">
@@ -8611,10 +8623,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>43133</v>
       </c>
-      <c r="B21" s="1" t="n">
+      <c r="B21" s="2" t="n">
         <v>43147</v>
       </c>
       <c r="C21" t="n">
@@ -8643,10 +8655,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>43217</v>
       </c>
-      <c r="B22" s="1" t="n">
+      <c r="B22" s="2" t="n">
         <v>43224</v>
       </c>
       <c r="C22" t="n">
@@ -8675,10 +8687,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>43312</v>
       </c>
-      <c r="B23" s="1" t="n">
+      <c r="B23" s="2" t="n">
         <v>43319</v>
       </c>
       <c r="C23" t="n">
@@ -8707,10 +8719,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>43404</v>
       </c>
-      <c r="B24" s="1" t="n">
+      <c r="B24" s="2" t="n">
         <v>43411</v>
       </c>
       <c r="C24" t="n">
@@ -8739,10 +8751,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>43504</v>
       </c>
-      <c r="B25" s="1" t="n">
+      <c r="B25" s="2" t="n">
         <v>43523</v>
       </c>
       <c r="C25" t="n">
@@ -8771,10 +8783,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>43581</v>
       </c>
-      <c r="B26" s="1" t="n">
+      <c r="B26" s="2" t="n">
         <v>43588</v>
       </c>
       <c r="C26" t="n">
@@ -8803,10 +8815,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>43675</v>
       </c>
-      <c r="B27" s="1" t="n">
+      <c r="B27" s="2" t="n">
         <v>43682</v>
       </c>
       <c r="C27" t="n">
@@ -8835,10 +8847,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>43767</v>
       </c>
-      <c r="B28" s="1" t="n">
+      <c r="B28" s="2" t="n">
         <v>43775</v>
       </c>
       <c r="C28" t="n">
@@ -8867,10 +8879,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>43861</v>
       </c>
-      <c r="B29" s="1" t="n">
+      <c r="B29" s="2" t="n">
         <v>43882</v>
       </c>
       <c r="C29" t="n">
@@ -8899,10 +8911,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>43951</v>
       </c>
-      <c r="B30" s="1" t="n">
+      <c r="B30" s="2" t="n">
         <v>43959</v>
       </c>
       <c r="C30" t="n">
@@ -8931,10 +8943,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>44040</v>
       </c>
-      <c r="B31" s="1" t="n">
+      <c r="B31" s="2" t="n">
         <v>44047</v>
       </c>
       <c r="C31" t="n">
@@ -8963,10 +8975,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>44131</v>
       </c>
-      <c r="B32" s="1" t="n">
+      <c r="B32" s="2" t="n">
         <v>44139</v>
       </c>
       <c r="C32" t="n">
@@ -8995,10 +9007,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>44227</v>
       </c>
-      <c r="B33" s="1" t="n">
+      <c r="B33" s="2" t="n">
         <v>44246</v>
       </c>
       <c r="C33" t="n">
@@ -9027,10 +9039,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>44314</v>
       </c>
-      <c r="B34" s="1" t="n">
+      <c r="B34" s="2" t="n">
         <v>44323</v>
       </c>
       <c r="C34" t="n">
@@ -9059,10 +9071,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>44403</v>
       </c>
-      <c r="B35" s="1" t="n">
+      <c r="B35" s="2" t="n">
         <v>44410</v>
       </c>
       <c r="C35" t="n">
@@ -9091,10 +9103,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>44494</v>
       </c>
-      <c r="B36" s="1" t="n">
+      <c r="B36" s="2" t="n">
         <v>44502</v>
       </c>
       <c r="C36" t="n">
@@ -9123,10 +9135,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>44592</v>
       </c>
-      <c r="B37" s="1" t="n">
+      <c r="B37" s="2" t="n">
         <v>44610</v>
       </c>
       <c r="C37" t="n">
@@ -9155,10 +9167,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>44678</v>
       </c>
-      <c r="B38" s="1" t="n">
+      <c r="B38" s="2" t="n">
         <v>44687</v>
       </c>
       <c r="C38" t="n">
@@ -9187,10 +9199,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>44769</v>
       </c>
-      <c r="B39" s="1" t="n">
+      <c r="B39" s="2" t="n">
         <v>44777</v>
       </c>
       <c r="C39" t="n">
@@ -9219,10 +9231,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>44860</v>
       </c>
-      <c r="B40" s="1" t="n">
+      <c r="B40" s="2" t="n">
         <v>44869</v>
       </c>
       <c r="C40" t="n">
@@ -9251,10 +9263,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>44957</v>
       </c>
-      <c r="B41" s="1" t="n">
+      <c r="B41" s="2" t="n">
         <v>44974</v>
       </c>
       <c r="C41" t="n">
@@ -9283,10 +9295,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>45041</v>
       </c>
-      <c r="B42" s="1" t="n">
+      <c r="B42" s="2" t="n">
         <v>45051</v>
       </c>
       <c r="C42" t="n">
@@ -9315,10 +9327,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>45138</v>
       </c>
-      <c r="B43" s="1" t="n">
+      <c r="B43" s="2" t="n">
         <v>45145</v>
       </c>
       <c r="C43" t="n">
@@ -9347,10 +9359,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>45226</v>
       </c>
-      <c r="B44" s="1" t="n">
+      <c r="B44" s="2" t="n">
         <v>45236</v>
       </c>
       <c r="C44" t="n">
@@ -9379,10 +9391,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>45322</v>
       </c>
-      <c r="B45" s="1" t="n">
+      <c r="B45" s="2" t="n">
         <v>45342</v>
       </c>
       <c r="C45" t="n">
@@ -9411,10 +9423,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>45407</v>
       </c>
-      <c r="B46" s="1" t="n">
+      <c r="B46" s="2" t="n">
         <v>45415</v>
       </c>
       <c r="C46" t="n">
@@ -9443,10 +9455,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>45502</v>
       </c>
-      <c r="B47" s="1" t="n">
+      <c r="B47" s="2" t="n">
         <v>45511</v>
       </c>
       <c r="C47" t="n">
@@ -9475,10 +9487,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>45593</v>
       </c>
-      <c r="B48" s="1" t="n">
+      <c r="B48" s="2" t="n">
         <v>45600</v>
       </c>
       <c r="C48" t="n">
@@ -9507,10 +9519,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>45688</v>
       </c>
-      <c r="B49" s="1" t="n">
+      <c r="B49" s="2" t="n">
         <v>45702</v>
       </c>
       <c r="C49" t="n">
@@ -9539,10 +9551,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>45777</v>
       </c>
-      <c r="B50" s="1" t="n">
+      <c r="B50" s="2" t="n">
         <v>45786</v>
       </c>
       <c r="C50" t="n">
@@ -9571,10 +9583,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>45867</v>
       </c>
-      <c r="B51" s="1" t="n">
+      <c r="B51" s="2" t="n">
         <v>45873</v>
       </c>
       <c r="C51" t="n">
@@ -9603,10 +9615,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>45957</v>
       </c>
-      <c r="B52" s="1" t="n">
+      <c r="B52" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="C52" t="n">
@@ -9635,10 +9647,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>46063</v>
       </c>
-      <c r="B53" s="1" t="n">
+      <c r="B53" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="C53" t="n">
@@ -9667,10 +9679,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="B54" s="1" t="n">
+      <c r="B54" s="2" t="n">
         <v>46150</v>
       </c>
       <c r="C54" t="n">
@@ -9699,10 +9711,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="B55" s="1" t="n">
+      <c r="B55" s="2" t="n">
         <v>46237</v>
       </c>
       <c r="C55" t="n">
@@ -9749,12 +9761,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>valor</t>
         </is>

</xml_diff>